<commit_message>
Implement Excel report formatting and insights sheet
</commit_message>
<xml_diff>
--- a/output/test_result (cn).xlsx
+++ b/output/test_result (cn).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ADInt\book-catalog-automation\output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08D95A93-C603-4262-825E-35EA2B21B0C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B978C48D-56BA-4D69-8E55-651DCBE9CF69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5712" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -37,9 +37,6 @@
     <t>conditions</t>
   </si>
   <si>
-    <t>name</t>
-  </si>
-  <si>
     <t>author</t>
   </si>
   <si>
@@ -182,14 +179,25 @@
   </si>
   <si>
     <t>price</t>
+  </si>
+  <si>
+    <t>title</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -246,15 +254,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -266,6 +265,15 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -585,352 +593,352 @@
     <col min="12" max="12" width="20.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" s="3" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="4" t="s">
+    <row r="1" spans="1:12" s="9" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="E1" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="F1" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="G1" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="H1" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="I1" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="J1" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="K1" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="K1" s="5" t="s">
+      <c r="L1" s="8" t="s">
         <v>9</v>
-      </c>
-      <c r="L1" s="5" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:12" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="6">
+      <c r="A2" s="3">
         <v>40001</v>
       </c>
-      <c r="B2" s="7">
+      <c r="B2" s="4">
         <v>70</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="C2" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2" s="4">
+        <v>1</v>
+      </c>
+      <c r="E2" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="D2" s="7">
-        <v>1</v>
-      </c>
-      <c r="E2" s="7" t="s">
+      <c r="F2" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="F2" s="6" t="s">
+      <c r="G2" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G2" s="7" t="s">
+      <c r="H2" s="4">
+        <v>221</v>
+      </c>
+      <c r="I2" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="H2" s="7">
-        <v>221</v>
-      </c>
-      <c r="I2" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="J2" s="7">
+      <c r="J2" s="4">
         <v>125</v>
       </c>
-      <c r="K2" s="8"/>
-      <c r="L2" s="9"/>
+      <c r="K2" s="5"/>
+      <c r="L2" s="6"/>
     </row>
     <row r="3" spans="1:12" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="6">
+      <c r="A3" s="3">
         <v>40002</v>
       </c>
-      <c r="B3" s="7">
+      <c r="B3" s="4">
         <v>70</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="C3" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3" s="4">
+        <v>1</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F3" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="D3" s="7">
-        <v>1</v>
-      </c>
-      <c r="E3" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="F3" s="6" t="s">
+      <c r="G3" s="4"/>
+      <c r="H3" s="4">
+        <v>214</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="J3" s="4">
+        <v>104</v>
+      </c>
+      <c r="K3" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="G3" s="7"/>
-      <c r="H3" s="7">
-        <v>214</v>
-      </c>
-      <c r="I3" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="J3" s="7">
-        <v>104</v>
-      </c>
-      <c r="K3" s="8" t="s">
+      <c r="L3" s="6" t="s">
         <v>18</v>
-      </c>
-      <c r="L3" s="9" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="4" spans="1:12" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="6">
+      <c r="A4" s="3">
         <v>40003</v>
       </c>
-      <c r="B4" s="7">
+      <c r="B4" s="4">
         <v>70</v>
       </c>
-      <c r="C4" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="D4" s="7">
+      <c r="C4" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D4" s="4">
         <v>1</v>
       </c>
-      <c r="E4" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="F4" s="6"/>
-      <c r="G4" s="7"/>
-      <c r="H4" s="7"/>
-      <c r="I4" s="7"/>
-      <c r="J4" s="7">
+      <c r="E4" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F4" s="3"/>
+      <c r="G4" s="4"/>
+      <c r="H4" s="4"/>
+      <c r="I4" s="4"/>
+      <c r="J4" s="4">
         <v>266</v>
       </c>
-      <c r="K4" s="8"/>
-      <c r="L4" s="9"/>
+      <c r="K4" s="5"/>
+      <c r="L4" s="6"/>
     </row>
     <row r="5" spans="1:12" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="6">
+      <c r="A5" s="3">
         <v>40004</v>
       </c>
-      <c r="B5" s="7">
+      <c r="B5" s="4">
         <v>70</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="C5" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D5" s="4">
+        <v>1</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F5" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="D5" s="7">
-        <v>1</v>
-      </c>
-      <c r="E5" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="F5" s="6" t="s">
+      <c r="G5" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="G5" s="7" t="s">
+      <c r="H5" s="4"/>
+      <c r="I5" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="H5" s="7"/>
-      <c r="I5" s="7" t="s">
+      <c r="J5" s="4"/>
+      <c r="K5" s="5"/>
+      <c r="L5" s="6" t="s">
         <v>24</v>
-      </c>
-      <c r="J5" s="7"/>
-      <c r="K5" s="8"/>
-      <c r="L5" s="9" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="6" spans="1:12" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="6">
+      <c r="A6" s="3">
         <v>40005</v>
       </c>
-      <c r="B6" s="7">
+      <c r="B6" s="4">
         <v>70</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D6" s="4">
+        <v>1</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F6" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="D6" s="7">
-        <v>1</v>
-      </c>
-      <c r="E6" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="F6" s="6" t="s">
+      <c r="G6" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="G6" s="7" t="s">
+      <c r="H6" s="4">
+        <v>202</v>
+      </c>
+      <c r="I6" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="H6" s="7">
-        <v>202</v>
-      </c>
-      <c r="I6" s="7" t="s">
+      <c r="J6" s="4">
+        <v>249</v>
+      </c>
+      <c r="K6" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="J6" s="7">
-        <v>249</v>
-      </c>
-      <c r="K6" s="8" t="s">
+      <c r="L6" s="6" t="s">
         <v>30</v>
-      </c>
-      <c r="L6" s="9" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="7" spans="1:12" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="6">
+      <c r="A7" s="3">
         <v>40006</v>
       </c>
-      <c r="B7" s="7">
+      <c r="B7" s="4">
         <v>70</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C7" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="D7" s="4">
+        <v>1</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F7" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="D7" s="7">
-        <v>1</v>
-      </c>
-      <c r="E7" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="F7" s="6" t="s">
+      <c r="G7" s="4"/>
+      <c r="H7" s="4"/>
+      <c r="I7" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="G7" s="7"/>
-      <c r="H7" s="7"/>
-      <c r="I7" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="J7" s="7">
+      <c r="J7" s="4">
         <v>449</v>
       </c>
-      <c r="K7" s="8"/>
-      <c r="L7" s="9"/>
+      <c r="K7" s="5"/>
+      <c r="L7" s="6"/>
     </row>
     <row r="8" spans="1:12" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="6">
+      <c r="A8" s="3">
         <v>40007</v>
       </c>
-      <c r="B8" s="7">
+      <c r="B8" s="4">
         <v>70</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="C8" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="D8" s="4">
+        <v>1</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F8" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="D8" s="7">
-        <v>1</v>
-      </c>
-      <c r="E8" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="F8" s="6" t="s">
+      <c r="G8" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="G8" s="7" t="s">
+      <c r="H8" s="4">
+        <v>268</v>
+      </c>
+      <c r="I8" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="H8" s="7">
-        <v>268</v>
-      </c>
-      <c r="I8" s="7" t="s">
+      <c r="J8" s="4">
+        <v>327</v>
+      </c>
+      <c r="K8" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="L8" s="6" t="s">
         <v>38</v>
-      </c>
-      <c r="J8" s="7">
-        <v>327</v>
-      </c>
-      <c r="K8" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="L8" s="9" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="9" spans="1:12" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="6">
+      <c r="A9" s="3">
         <v>40008</v>
       </c>
-      <c r="B9" s="7">
+      <c r="B9" s="4">
         <v>70</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="C9" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="D9" s="4">
+        <v>1</v>
+      </c>
+      <c r="E9" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="D9" s="7">
-        <v>1</v>
-      </c>
-      <c r="E9" s="7" t="s">
+      <c r="F9" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="F9" s="6" t="s">
+      <c r="G9" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="G9" s="7" t="s">
+      <c r="H9" s="4">
+        <v>117</v>
+      </c>
+      <c r="I9" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="H9" s="7">
-        <v>117</v>
-      </c>
-      <c r="I9" s="7" t="s">
+      <c r="J9" s="4">
+        <v>178</v>
+      </c>
+      <c r="K9" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="J9" s="7">
-        <v>178</v>
-      </c>
-      <c r="K9" s="8" t="s">
+      <c r="L9" s="6" t="s">
         <v>45</v>
-      </c>
-      <c r="L9" s="9" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="10" spans="1:12" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="6">
+      <c r="A10" s="3">
         <v>40009</v>
       </c>
-      <c r="B10" s="7">
+      <c r="B10" s="4">
         <v>70</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="C10" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="D10" s="4">
+        <v>1</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="F10" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="D10" s="7">
-        <v>1</v>
-      </c>
-      <c r="E10" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="F10" s="6" t="s">
+      <c r="G10" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="G10" s="7" t="s">
+      <c r="H10" s="4">
+        <v>54</v>
+      </c>
+      <c r="I10" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="H10" s="7">
-        <v>54</v>
-      </c>
-      <c r="I10" s="7" t="s">
+      <c r="J10" s="4">
+        <v>288</v>
+      </c>
+      <c r="K10" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="J10" s="7">
-        <v>288</v>
-      </c>
-      <c r="K10" s="8" t="s">
+      <c r="L10" s="6" t="s">
         <v>51</v>
-      </c>
-      <c r="L10" s="9" t="s">
-        <v>52</v>
       </c>
     </row>
   </sheetData>

</xml_diff>